<commit_message>
latest updated latest updated 1 latest updated 2
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -16,6 +16,47 @@
     </ext>
   </extLst>
 </workbook>
+</file>
+
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+  <si>
+    <t>ID</t>
+  </si>
+  <si>
+    <t>NAME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CITY </t>
+  </si>
+  <si>
+    <t>SALARY</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>B</t>
+  </si>
+  <si>
+    <t>C</t>
+  </si>
+  <si>
+    <t>D</t>
+  </si>
+  <si>
+    <t>X</t>
+  </si>
+  <si>
+    <t>Y</t>
+  </si>
+  <si>
+    <t>Z</t>
+  </si>
+  <si>
+    <t>O</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -331,9 +372,80 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2">
+        <v>156516</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3">
+        <v>64846</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D4">
+        <v>68464646</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D5">
+        <v>6848643</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>